<commit_message>
fix(original-pirate): migrate source candidates to v39
</commit_message>
<xml_diff>
--- a/xlsx/candidates/original_pirate_cannonball_none.xlsx
+++ b/xlsx/candidates/original_pirate_cannonball_none.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S4"/>
+  <dimension ref="A1:T4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -443,75 +443,80 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>availability</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>base_quality</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>quality</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>buy_price</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>sell_price</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>activation_mode</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>cooldown_ticks</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>crit_chance_bps</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>ammo_enabled</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>ammo_initial</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>ammo_maximum</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>item_skill_id</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>starter_instance_id</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>starter_location</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>starter_start_slot</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>catalog_status</t>
         </is>
@@ -528,7 +533,6 @@
           <t>炮弹（原版未附魔候选）</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>1</t>
@@ -536,67 +540,70 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>run_acquirable</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>silver</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>silver</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>passive</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>skill_bazaar_cannonball</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>candidate_cannonball_silver</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>stash</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>formal</t>
         </is>
@@ -613,7 +620,6 @@
           <t>炮弹（原版未附魔候选）</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>1</t>
@@ -621,59 +627,60 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>run_acquirable</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>silver</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>gold</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>passive</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>skill_bazaar_cannonball</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>formal</t>
         </is>
@@ -690,7 +697,6 @@
           <t>炮弹（原版未附魔候选）</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>1</t>
@@ -698,59 +704,60 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>run_acquirable</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>silver</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>diamond</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>passive</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>skill_bazaar_cannonball</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>formal</t>
         </is>
@@ -823,8 +830,6 @@
           <t>装备时，己方最大弹药大于零的物品增加最大弹药；不补充当前弹药。仅未附魔候选。</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>aura_bazaar_cannonball_silver,aura_bazaar_cannonball_gold,aura_bazaar_cannonball_diamond</t>
@@ -1068,7 +1073,6 @@
           <t>friendly_ammo_items</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>false</t>
@@ -1084,7 +1088,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
           <t>formal</t>
@@ -1122,7 +1125,6 @@
           <t>friendly_ammo_items</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>false</t>
@@ -1138,7 +1140,6 @@
           <t>2</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>formal</t>
@@ -1176,7 +1177,6 @@
           <t>friendly_ammo_items</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>false</t>
@@ -1192,7 +1192,6 @@
           <t>3</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
           <t>formal</t>

</xml_diff>